<commit_message>
fix an issue in distance-based scoring
</commit_message>
<xml_diff>
--- a/llm_labeling/code2text_python_rating.xlsx
+++ b/llm_labeling/code2text_python_rating.xlsx
@@ -510,7 +510,7 @@
         <v>0.9355779686079343</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2" t="n">
         <v>1.008166070895517</v>
@@ -549,7 +549,7 @@
         <v>1.007200515691478</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -588,7 +588,7 @@
         <v>0.9280379612394892</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
         <v>0.8593372714230572</v>
@@ -627,7 +627,7 @@
         <v>0.8035881040050555</v>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J5" t="n">
         <v>1.650987722989433</v>
@@ -666,7 +666,7 @@
         <v>0.7465580872262197</v>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" t="n">
         <v>1.062577052993187</v>
@@ -705,7 +705,7 @@
         <v>0.6872661189957208</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
         <v>1.20566018689926</v>
@@ -744,7 +744,7 @@
         <v>0.6955043614872732</v>
       </c>
       <c r="I8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
         <v>1.315279920511133</v>
@@ -783,7 +783,7 @@
         <v>0.3552721923209445</v>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
         <v>2.50319294874323</v>
@@ -822,7 +822,7 @@
         <v>0.9216283858270756</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" t="n">
         <v>0.8284204781041018</v>
@@ -861,7 +861,7 @@
         <v>0.9059732599740568</v>
       </c>
       <c r="I11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>1.177658947627176</v>
@@ -900,7 +900,7 @@
         <v>0.9170126222558316</v>
       </c>
       <c r="I12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0.3590524547360447</v>
@@ -939,7 +939,7 @@
         <v>0.6400204942641929</v>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" t="n">
         <v>1.559584333403506</v>
@@ -978,7 +978,7 @@
         <v>1.302798802626917</v>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0.1310828260534545</v>
@@ -1017,7 +1017,7 @@
         <v>1.076215402714742</v>
       </c>
       <c r="I15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J15" t="n">
         <v>0.450388625059611</v>
@@ -1056,7 +1056,7 @@
         <v>0.7464942484767676</v>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J16" t="n">
         <v>1.077456194435146</v>
@@ -1095,7 +1095,7 @@
         <v>0.5697936236071852</v>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
         <v>1.656014595354423</v>
@@ -1134,7 +1134,7 @@
         <v>0.9881054343682446</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
         <v>0.8211119422493731</v>
@@ -1173,7 +1173,7 @@
         <v>0.8051384213679031</v>
       </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J19" t="n">
         <v>0.8842147704847014</v>
@@ -1212,7 +1212,7 @@
         <v>0.9711673315527326</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
         <v>0.2883534452447986</v>
@@ -1251,7 +1251,7 @@
         <v>0.8437938048446951</v>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
         <v>0.9741696147001039</v>
@@ -1290,7 +1290,7 @@
         <v>0.8628233033391974</v>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J22" t="n">
         <v>1.789856946466333</v>
@@ -1329,7 +1329,7 @@
         <v>0.6980982977874831</v>
       </c>
       <c r="I23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
         <v>1.2824649352103</v>

</xml_diff>